<commit_message>
new dmcar development adding keys to model serialisation
</commit_message>
<xml_diff>
--- a/tests/serialisation_templates/datamodel/datamodel_template_v1.xlsx
+++ b/tests/serialisation_templates/datamodel/datamodel_template_v1.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Definitions!$A$1:$E$44</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Example(Library Model)'!$A$1:$AS$20</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Example(Library Model)'!$A$1:$AT$22</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="242">
   <si>
     <t xml:space="preserve">SubjectArea</t>
   </si>
@@ -209,12 +209,21 @@
     <t xml:space="preserve">The (primary) key used to reference the target entity by this relationship</t>
   </si>
   <si>
+    <t xml:space="preserve">RelationshipNamespace</t>
+  </si>
+  <si>
     <t xml:space="preserve">SourceRoleEntity</t>
   </si>
   <si>
+    <t xml:space="preserve">TargetEntityNamespace</t>
+  </si>
+  <si>
     <t xml:space="preserve">TargetRoleEntity</t>
   </si>
   <si>
+    <t xml:space="preserve">Base</t>
+  </si>
+  <si>
     <t xml:space="preserve">Party</t>
   </si>
   <si>
@@ -278,7 +287,7 @@
     <t xml:space="preserve">PartyRoleIdentifier</t>
   </si>
   <si>
-    <t xml:space="preserve">Person Role Identifier</t>
+    <t xml:space="preserve">Party Role Identifier</t>
   </si>
   <si>
     <t xml:space="preserve">An internal identifier used to reference a specific Person-Role Context.</t>
@@ -407,9 +416,6 @@
     <t xml:space="preserve">assignsAuthorshipBy</t>
   </si>
   <si>
-    <t xml:space="preserve">FK-Author</t>
-  </si>
-  <si>
     <t xml:space="preserve">Library</t>
   </si>
   <si>
@@ -494,13 +500,40 @@
     <t xml:space="preserve">LibraryMembershipIdentifier</t>
   </si>
   <si>
-    <t xml:space="preserve">:ibrary Membership Identifier</t>
+    <t xml:space="preserve">Library Membership Identifier</t>
   </si>
   <si>
     <t xml:space="preserve">An internal identifier used to reference a specific membership relation between a Library and a person-acting as a member.</t>
   </si>
   <si>
     <t xml:space="preserve">Primary Key on LibraryMembership</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A reference to the Library that manages the Membership</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Membership-Library</t>
+  </si>
+  <si>
+    <t xml:space="preserve">withLibrary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">managesMembership</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A reference to the PartyRole that identifies the member</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Membership-PartyRole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Member</t>
+  </si>
+  <si>
+    <t xml:space="preserve">forMember</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hasMembership</t>
   </si>
   <si>
     <t xml:space="preserve">Loan</t>
@@ -1421,15 +1454,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:XFD26"/>
+  <dimension ref="A1:AT28"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.18"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="21.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="23.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="25.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16.73"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16.73"/>
@@ -1451,25 +1484,26 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="27.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="24.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="23.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="25.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="17.15"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="31" min="31" style="1" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="0" width="16.59"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="20.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="0" width="16.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="0" width="14.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="0" width="18.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="0" width="20.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="0" width="16.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="0" width="14.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="0" width="10.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="0" width="15.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="0" width="14.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="0" width="18.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="0" width="20.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="29" style="0" width="25.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="0" width="17.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="1" width="25.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="16.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="0" width="20.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="0" width="18.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="0" width="16.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="0" width="14.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="0" width="18.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="0" width="20.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="0" width="16.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="0" width="14.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="0" width="10.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="0" width="15.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="0" width="14.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="0" width="18.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="0" width="20.22"/>
   </cols>
   <sheetData>
-    <row r="1" s="2" customFormat="true" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" s="2" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
@@ -1555,1160 +1589,1312 @@
         <v>51</v>
       </c>
       <c r="AC1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AE1" s="3" t="s">
+      <c r="AF1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AG1" s="2" t="s">
-        <v>60</v>
-      </c>
       <c r="AH1" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="AI1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AL1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AM1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="AM1" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="AN1" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="AO1" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="AP1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="AP1" s="2" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="AQ1" s="2" t="s">
+      <c r="AR1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="AR1" s="2" t="s">
+      <c r="AS1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AS1" s="2" t="s">
+      <c r="AT1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="XFD1" s="0"/>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N2" s="0" t="s">
+        <v>64</v>
+      </c>
       <c r="O2" s="0" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="P2" s="0" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="Q2" s="1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="R2" s="0" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="S2" s="0" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="T2" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="U2" s="0" t="n">
         <v>1</v>
       </c>
       <c r="V2" s="0" t="s">
+        <v>70</v>
+      </c>
+      <c r="W2" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="X2" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y2" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="Z2" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="AB2" s="0" t="s">
         <v>67</v>
       </c>
-      <c r="W2" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="X2" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="Y2" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="Z2" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="AA2" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="AB2" s="0" t="s">
-        <v>64</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N3" s="0" t="s">
+        <v>64</v>
+      </c>
       <c r="O3" s="0" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="P3" s="0" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="R3" s="0" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="S3" s="0" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="T3" s="1" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="U3" s="0" t="n">
         <v>1</v>
       </c>
       <c r="V3" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="W3" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="X3" s="0" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="Y3" s="0" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="Z3" s="0" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="AA3" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="AB3" s="0" t="s">
         <v>78</v>
       </c>
-      <c r="AB3" s="0" t="s">
-        <v>75</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N4" s="0" t="s">
+        <v>64</v>
+      </c>
       <c r="O4" s="0" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="P4" s="0" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="R4" s="0" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="S4" s="0" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="U4" s="0" t="n">
         <v>1</v>
       </c>
       <c r="V4" s="0" t="s">
+        <v>70</v>
+      </c>
+      <c r="W4" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="X4" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y4" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="Z4" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA4" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="AB4" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="AF4" s="0"/>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N5" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="O5" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="P5" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="R5" s="0" t="s">
         <v>67</v>
       </c>
-      <c r="W4" s="0" t="s">
+      <c r="S5" s="0" t="s">
         <v>68</v>
-      </c>
-      <c r="X4" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="Y4" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="Z4" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="AA4" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="AB4" s="0" t="s">
-        <v>82</v>
-      </c>
-      <c r="AE4" s="0"/>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O5" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="P5" s="0" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q5" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="R5" s="0" t="s">
-        <v>64</v>
-      </c>
-      <c r="S5" s="0" t="s">
-        <v>65</v>
       </c>
       <c r="U5" s="0" t="n">
         <v>2</v>
       </c>
       <c r="V5" s="0" t="s">
+        <v>70</v>
+      </c>
+      <c r="W5" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="X5" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y5" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z5" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="AB5" s="0" t="s">
         <v>67</v>
       </c>
-      <c r="W5" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="X5" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="Y5" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="Z5" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="AB5" s="0" t="s">
-        <v>64</v>
-      </c>
       <c r="AC5" s="0" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="AD5" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="AE5" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="AH5" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AI5" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="AJ5" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="AK5" s="0" t="s">
         <v>89</v>
       </c>
-      <c r="AG5" s="0" t="s">
+      <c r="AL5" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AM5" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN5" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AO5" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="AP5" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="AQ5" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="AR5" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="AS5" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AT5" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N6" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="O6" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="P6" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="Q6" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="R6" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="S6" s="0" t="s">
         <v>79</v>
-      </c>
-      <c r="AH5" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="AI5" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="AJ5" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="AK5" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AL5" s="0" t="s">
-        <v>91</v>
-      </c>
-      <c r="AN5" s="0" t="s">
-        <v>62</v>
-      </c>
-      <c r="AO5" s="0" t="s">
-        <v>92</v>
-      </c>
-      <c r="AP5" s="0" t="s">
-        <v>92</v>
-      </c>
-      <c r="AQ5" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="AR5" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AS5" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O6" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="P6" s="0" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q6" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="R6" s="0" t="s">
-        <v>75</v>
-      </c>
-      <c r="S6" s="0" t="s">
-        <v>76</v>
       </c>
       <c r="U6" s="0" t="n">
         <v>3</v>
       </c>
       <c r="V6" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="W6" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="X6" s="0" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="Y6" s="0" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="Z6" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="AB6" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="AC6" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AD6" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="AE6" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="AH6" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AI6" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="AJ6" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="AK6" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="AL6" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AM6" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="AB6" s="0" t="s">
-        <v>75</v>
-      </c>
-      <c r="AC6" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="AD6" s="0" t="s">
-        <v>96</v>
-      </c>
-      <c r="AG6" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="AH6" s="0" t="s">
-        <v>97</v>
-      </c>
-      <c r="AI6" s="0" t="s">
-        <v>97</v>
-      </c>
-      <c r="AJ6" s="0" t="s">
-        <v>93</v>
-      </c>
-      <c r="AK6" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AL6" s="0" t="s">
-        <v>91</v>
-      </c>
       <c r="AN6" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AO6" s="0" t="s">
+        <v>76</v>
+      </c>
+      <c r="AP6" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="AQ6" s="0" t="s">
+        <v>76</v>
+      </c>
+      <c r="AR6" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="AO6" s="0" t="s">
-        <v>98</v>
-      </c>
-      <c r="AP6" s="0" t="s">
-        <v>73</v>
-      </c>
-      <c r="AQ6" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="AR6" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AS6" s="0" t="n">
+      <c r="AS6" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AT6" s="0" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N7" s="0" t="s">
+        <v>64</v>
+      </c>
       <c r="O7" s="0" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="P7" s="0" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="R7" s="0" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="S7" s="0" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="T7" s="1" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="U7" s="0" t="n">
         <v>1</v>
       </c>
       <c r="V7" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="W7" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="X7" s="0" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="Y7" s="0" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="Z7" s="0" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="AA7" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="AB7" s="0" t="s">
         <v>104</v>
       </c>
-      <c r="AB7" s="0" t="s">
-        <v>101</v>
-      </c>
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N8" s="0" t="s">
+        <v>64</v>
+      </c>
       <c r="O8" s="0" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P8" s="0" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="R8" s="0" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="S8" s="0" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="U8" s="0" t="n">
         <v>1</v>
       </c>
       <c r="V8" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="W8" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="X8" s="0" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="Y8" s="0" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="Z8" s="0" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="AA8" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="AB8" s="0" t="s">
         <v>111</v>
       </c>
-      <c r="AB8" s="0" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N9" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="O9" s="0" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O9" s="0" t="s">
+      <c r="P9" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="Q9" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="R9" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="S9" s="0" t="s">
         <v>105</v>
       </c>
-      <c r="P9" s="0" t="s">
-        <v>106</v>
-      </c>
-      <c r="Q9" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="R9" s="0" t="s">
-        <v>101</v>
-      </c>
-      <c r="S9" s="0" t="s">
-        <v>102</v>
-      </c>
       <c r="T9" s="1" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="U9" s="0" t="n">
         <v>2</v>
       </c>
       <c r="V9" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="W9" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="X9" s="0" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="Y9" s="0" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="Z9" s="0" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AB9" s="0" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="AC9" s="0" t="s">
-        <v>115</v>
+        <v>64</v>
       </c>
       <c r="AD9" s="0" t="s">
-        <v>99</v>
-      </c>
-      <c r="AG9" s="0" t="s">
-        <v>105</v>
+        <v>118</v>
+      </c>
+      <c r="AE9" s="0" t="s">
+        <v>102</v>
       </c>
       <c r="AH9" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="AI9" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="AJ9" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="AK9" s="0" t="s">
         <v>116</v>
       </c>
-      <c r="AI9" s="0" t="s">
-        <v>116</v>
-      </c>
-      <c r="AJ9" s="0" t="s">
-        <v>113</v>
-      </c>
-      <c r="AL9" s="0" t="s">
-        <v>91</v>
+      <c r="AM9" s="0" t="s">
+        <v>94</v>
       </c>
       <c r="AN9" s="0" t="s">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="AO9" s="0" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="AP9" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="AQ9" s="0" t="s">
-        <v>70</v>
+        <v>121</v>
       </c>
       <c r="AR9" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AS9" s="0" t="n">
+        <v>73</v>
+      </c>
+      <c r="AS9" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AT9" s="0" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N10" s="0" t="s">
+        <v>64</v>
+      </c>
       <c r="O10" s="0" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P10" s="0" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="R10" s="0" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="S10" s="0" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="T10" s="1" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="U10" s="0" t="n">
         <v>3</v>
       </c>
       <c r="V10" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="W10" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="X10" s="0" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="Y10" s="0" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="Z10" s="0" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="AB10" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="AC10" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AD10" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="AE10" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="AH10" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="AI10" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ10" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="AK10" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="AM10" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN10" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AO10" s="0" t="s">
         <v>82</v>
       </c>
-      <c r="AC10" s="0" t="s">
-        <v>123</v>
-      </c>
-      <c r="AD10" s="0" t="s">
-        <v>124</v>
-      </c>
-      <c r="AG10" s="0" t="s">
-        <v>105</v>
-      </c>
-      <c r="AH10" s="0" t="s">
-        <v>125</v>
-      </c>
-      <c r="AI10" s="0" t="s">
-        <v>125</v>
-      </c>
-      <c r="AJ10" s="0" t="s">
-        <v>126</v>
-      </c>
-      <c r="AL10" s="0" t="s">
-        <v>91</v>
-      </c>
-      <c r="AN10" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="AO10" s="0" t="s">
-        <v>124</v>
-      </c>
       <c r="AP10" s="0" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="AQ10" s="0" t="s">
-        <v>70</v>
+        <v>127</v>
       </c>
       <c r="AR10" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AS10" s="0" t="n">
+        <v>73</v>
+      </c>
+      <c r="AS10" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AT10" s="0" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N11" s="0" t="s">
+        <v>64</v>
+      </c>
       <c r="O11" s="0" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="P11" s="0" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="R11" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="S11" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="T11" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="U11" s="0" t="n">
         <v>1</v>
       </c>
       <c r="V11" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="W11" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="X11" s="0" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="Y11" s="0" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="Z11" s="0" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="AA11" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="AB11" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N12" s="0" t="s">
+        <v>64</v>
+      </c>
       <c r="O12" s="0" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="P12" s="0" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="R12" s="0" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="S12" s="0" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="T12" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="U12" s="0" t="n">
         <v>1</v>
       </c>
       <c r="V12" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="W12" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="X12" s="0" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="Y12" s="0" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="Z12" s="0" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="AA12" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="AB12" s="0" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N13" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="O13" s="0" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O13" s="0" t="s">
-        <v>133</v>
-      </c>
       <c r="P13" s="0" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="Q13" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="R13" s="0" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="S13" s="0" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="T13" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="U13" s="0" t="n">
         <v>2</v>
       </c>
       <c r="V13" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="W13" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="X13" s="0" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="Y13" s="0" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="Z13" s="0" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AB13" s="0" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="AC13" s="0" t="s">
-        <v>140</v>
+        <v>64</v>
       </c>
       <c r="AD13" s="0" t="s">
-        <v>141</v>
-      </c>
-      <c r="AG13" s="0" t="s">
-        <v>133</v>
+        <v>142</v>
+      </c>
+      <c r="AE13" s="0" t="s">
+        <v>143</v>
       </c>
       <c r="AH13" s="0" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="AI13" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="AJ13" s="0" t="s">
-        <v>113</v>
+        <v>145</v>
       </c>
       <c r="AK13" s="0" t="s">
-        <v>69</v>
+        <v>116</v>
       </c>
       <c r="AL13" s="0" t="s">
-        <v>91</v>
+        <v>72</v>
+      </c>
+      <c r="AM13" s="0" t="s">
+        <v>94</v>
       </c>
       <c r="AN13" s="0" t="s">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="AO13" s="0" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="AP13" s="0" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="AQ13" s="0" t="s">
-        <v>70</v>
+        <v>102</v>
       </c>
       <c r="AR13" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AS13" s="0" t="n">
+        <v>73</v>
+      </c>
+      <c r="AS13" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AT13" s="0" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N14" s="0" t="s">
+        <v>64</v>
+      </c>
       <c r="O14" s="0" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="P14" s="0" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="Q14" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="R14" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="S14" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="T14" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="U14" s="0" t="n">
         <v>3</v>
       </c>
       <c r="V14" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="W14" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="X14" s="0" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="Y14" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="Z14" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="AB14" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="AC14" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AD14" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="AE14" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="AH14" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI14" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="AJ14" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="AK14" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="AL14" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AM14" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN14" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AO14" s="0" t="s">
         <v>129</v>
       </c>
-      <c r="AC14" s="0" t="s">
-        <v>147</v>
-      </c>
-      <c r="AD14" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="AG14" s="0" t="s">
-        <v>133</v>
-      </c>
-      <c r="AH14" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="AI14" s="0" t="s">
-        <v>149</v>
-      </c>
-      <c r="AJ14" s="0" t="s">
-        <v>145</v>
-      </c>
-      <c r="AK14" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AL14" s="0" t="s">
-        <v>91</v>
-      </c>
-      <c r="AN14" s="0" t="s">
-        <v>127</v>
-      </c>
-      <c r="AO14" s="0" t="s">
-        <v>150</v>
-      </c>
       <c r="AP14" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="AQ14" s="0" t="s">
-        <v>70</v>
+        <v>152</v>
       </c>
       <c r="AR14" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AS14" s="0" t="n">
+        <v>73</v>
+      </c>
+      <c r="AS14" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AT14" s="0" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N15" s="0" t="s">
+        <v>64</v>
+      </c>
       <c r="O15" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="P15" s="0" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="Q15" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="R15" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="S15" s="0" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="T15" s="1" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="U15" s="0" t="n">
         <v>1</v>
       </c>
       <c r="V15" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="W15" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="X15" s="0" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="Y15" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="Z15" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA15" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="AB15" s="0" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N16" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="O16" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="P16" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="Q16" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="R16" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="S16" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="T16" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="U16" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="V16" s="0" t="s">
         <v>70</v>
       </c>
-      <c r="Z15" s="0" t="s">
+      <c r="W16" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="AA15" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="AB15" s="0" t="s">
+      <c r="X16" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y16" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="Z16" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="AB16" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="AC16" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AD16" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="AE16" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="AH16" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="AI16" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="AJ16" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="AK16" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="AL16" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AM16" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN16" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AO16" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="AP16" s="0" t="s">
+        <v>163</v>
+      </c>
+      <c r="AQ16" s="0" t="s">
+        <v>163</v>
+      </c>
+      <c r="AR16" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="AS16" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AT16" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N17" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="O17" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="P17" s="0" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O16" s="0" t="s">
-        <v>158</v>
-      </c>
-      <c r="P16" s="0" t="s">
-        <v>158</v>
-      </c>
-      <c r="Q16" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="R16" s="0" t="s">
-        <v>160</v>
-      </c>
-      <c r="S16" s="0" t="s">
-        <v>161</v>
-      </c>
-      <c r="T16" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="U16" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="V16" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="W16" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="X16" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="Y16" s="0" t="s">
+      <c r="Q17" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="R17" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="S17" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="T17" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="U17" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="V17" s="0" t="s">
         <v>70</v>
       </c>
-      <c r="Z16" s="0" t="s">
+      <c r="W17" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="AA16" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="AB16" s="0" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O17" s="0" t="s">
-        <v>158</v>
-      </c>
-      <c r="P17" s="0" t="s">
-        <v>158</v>
-      </c>
-      <c r="Q17" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="R17" s="0" t="s">
-        <v>164</v>
-      </c>
-      <c r="S17" s="0" t="s">
+      <c r="X17" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y17" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="Z17" s="0" t="s">
+        <v>125</v>
+      </c>
+      <c r="AB17" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="AC17" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AD17" s="0" t="s">
         <v>165</v>
       </c>
-      <c r="T17" s="1" t="s">
+      <c r="AE17" s="0" t="s">
         <v>166</v>
       </c>
-      <c r="U17" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="V17" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="W17" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="X17" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="Y17" s="0" t="s">
-        <v>167</v>
-      </c>
-      <c r="Z17" s="0" t="s">
-        <v>168</v>
-      </c>
-      <c r="AB17" s="0" t="s">
-        <v>164</v>
-      </c>
-      <c r="AC17" s="0" t="s">
-        <v>169</v>
-      </c>
-      <c r="AG17" s="0" t="s">
-        <v>158</v>
-      </c>
       <c r="AH17" s="0" t="s">
-        <v>170</v>
+        <v>153</v>
       </c>
       <c r="AI17" s="0" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="AJ17" s="0" t="s">
         <v>167</v>
       </c>
       <c r="AK17" s="0" t="s">
-        <v>69</v>
+        <v>124</v>
       </c>
       <c r="AL17" s="0" t="s">
-        <v>91</v>
+        <v>72</v>
+      </c>
+      <c r="AM17" s="0" t="s">
+        <v>94</v>
       </c>
       <c r="AN17" s="0" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
       <c r="AO17" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="AP17" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="AQ17" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="AR17" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="AS17" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AT17" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N18" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="O18" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="P18" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="Q18" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="R18" s="0" t="s">
+        <v>171</v>
+      </c>
+      <c r="S18" s="0" t="s">
         <v>172</v>
       </c>
-      <c r="AP17" s="0" t="s">
+      <c r="T18" s="1" t="s">
         <v>173</v>
-      </c>
-      <c r="AQ17" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="AR17" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AS17" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O18" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="P18" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="Q18" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="R18" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="S18" s="0" t="s">
-        <v>178</v>
-      </c>
-      <c r="T18" s="1" t="s">
-        <v>179</v>
       </c>
       <c r="U18" s="0" t="n">
         <v>1</v>
       </c>
       <c r="V18" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="W18" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="X18" s="0" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="Y18" s="0" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="Z18" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA18" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="AB18" s="0" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N19" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="O19" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="P19" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="Q19" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="R19" s="0" t="s">
+        <v>175</v>
+      </c>
+      <c r="S19" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="T19" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="AA18" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="AB18" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O19" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="P19" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="Q19" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="R19" s="0" t="s">
-        <v>160</v>
-      </c>
-      <c r="S19" s="0" t="s">
-        <v>161</v>
-      </c>
-      <c r="T19" s="1" t="s">
-        <v>181</v>
       </c>
       <c r="U19" s="0" t="n">
         <v>2</v>
       </c>
       <c r="V19" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="W19" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="X19" s="0" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="Y19" s="0" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="Z19" s="0" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="AB19" s="0" t="s">
-        <v>160</v>
+        <v>175</v>
       </c>
       <c r="AC19" s="0" t="s">
-        <v>184</v>
+        <v>64</v>
       </c>
       <c r="AD19" s="0" t="s">
-        <v>185</v>
-      </c>
-      <c r="AG19" s="0" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="AH19" s="0" t="s">
-        <v>186</v>
+        <v>169</v>
       </c>
       <c r="AI19" s="0" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="AJ19" s="0" t="s">
         <v>182</v>
       </c>
       <c r="AK19" s="0" t="s">
-        <v>69</v>
+        <v>178</v>
       </c>
       <c r="AL19" s="0" t="s">
-        <v>91</v>
+        <v>72</v>
+      </c>
+      <c r="AM19" s="0" t="s">
+        <v>94</v>
       </c>
       <c r="AN19" s="0" t="s">
-        <v>158</v>
+        <v>64</v>
       </c>
       <c r="AO19" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="AP19" s="0" t="s">
+        <v>183</v>
+      </c>
+      <c r="AQ19" s="0" t="s">
+        <v>184</v>
+      </c>
+      <c r="AR19" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="AS19" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AT19" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N20" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="O20" s="0" t="s">
+        <v>185</v>
+      </c>
+      <c r="P20" s="0" t="s">
+        <v>186</v>
+      </c>
+      <c r="Q20" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="R20" s="0" t="s">
         <v>188</v>
-      </c>
-      <c r="AP19" s="0" t="s">
-        <v>188</v>
-      </c>
-      <c r="AQ19" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="AR19" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AS19" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O20" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="P20" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="Q20" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="R20" s="0" t="s">
-        <v>135</v>
       </c>
       <c r="S20" s="0" t="s">
         <v>189</v>
@@ -2717,428 +2903,609 @@
         <v>190</v>
       </c>
       <c r="U20" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="V20" s="0" t="s">
+        <v>70</v>
+      </c>
+      <c r="W20" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="X20" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y20" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="Z20" s="0" t="s">
+        <v>188</v>
+      </c>
+      <c r="AA20" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="AB20" s="0" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N21" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="O21" s="0" t="s">
+        <v>185</v>
+      </c>
+      <c r="P21" s="0" t="s">
+        <v>186</v>
+      </c>
+      <c r="Q21" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="R21" s="0" t="s">
+        <v>171</v>
+      </c>
+      <c r="S21" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="T21" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="U21" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="V21" s="0" t="s">
+        <v>70</v>
+      </c>
+      <c r="W21" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="X21" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y21" s="0" t="s">
+        <v>193</v>
+      </c>
+      <c r="Z21" s="0" t="s">
+        <v>194</v>
+      </c>
+      <c r="AB21" s="0" t="s">
+        <v>171</v>
+      </c>
+      <c r="AC21" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AD21" s="0" t="s">
+        <v>195</v>
+      </c>
+      <c r="AE21" s="0" t="s">
+        <v>196</v>
+      </c>
+      <c r="AH21" s="0" t="s">
+        <v>185</v>
+      </c>
+      <c r="AI21" s="0" t="s">
+        <v>197</v>
+      </c>
+      <c r="AJ21" s="0" t="s">
+        <v>198</v>
+      </c>
+      <c r="AK21" s="0" t="s">
+        <v>193</v>
+      </c>
+      <c r="AL21" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AM21" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN21" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AO21" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="AP21" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="AQ21" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="AR21" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="AS21" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AT21" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N22" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="O22" s="0" t="s">
+        <v>185</v>
+      </c>
+      <c r="P22" s="0" t="s">
+        <v>186</v>
+      </c>
+      <c r="Q22" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="R22" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="S22" s="0" t="s">
+        <v>200</v>
+      </c>
+      <c r="T22" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="U22" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="V20" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="W20" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="X20" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="Y20" s="0" t="s">
-        <v>191</v>
-      </c>
-      <c r="Z20" s="0" t="s">
-        <v>192</v>
-      </c>
-      <c r="AB20" s="0" t="s">
+      <c r="V22" s="0" t="s">
+        <v>70</v>
+      </c>
+      <c r="W22" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="X22" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y22" s="0" t="s">
+        <v>202</v>
+      </c>
+      <c r="Z22" s="0" t="s">
+        <v>203</v>
+      </c>
+      <c r="AB22" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="AC22" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AD22" s="0" t="s">
+        <v>204</v>
+      </c>
+      <c r="AE22" s="0" t="s">
         <v>135</v>
       </c>
-      <c r="AC20" s="0" t="s">
-        <v>193</v>
-      </c>
-      <c r="AD20" s="0" t="s">
-        <v>133</v>
-      </c>
-      <c r="AG20" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="AH20" s="0" t="s">
-        <v>194</v>
-      </c>
-      <c r="AI20" s="0" t="s">
-        <v>194</v>
-      </c>
-      <c r="AJ20" s="0" t="s">
-        <v>191</v>
-      </c>
-      <c r="AK20" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AL20" s="0" t="s">
-        <v>91</v>
-      </c>
-      <c r="AN20" s="0" t="s">
-        <v>133</v>
-      </c>
-      <c r="AO20" s="0" t="s">
-        <v>195</v>
-      </c>
-      <c r="AP20" s="0" t="s">
-        <v>196</v>
-      </c>
-      <c r="AQ20" s="0" t="s">
+      <c r="AH22" s="0" t="s">
+        <v>185</v>
+      </c>
+      <c r="AI22" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="AJ22" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="AK22" s="0" t="s">
+        <v>202</v>
+      </c>
+      <c r="AL22" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AM22" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN22" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AO22" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="AP22" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="AQ22" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="AR22" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="AS22" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AT22" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N23" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="O23" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="P23" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="Q23" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="R23" s="0" t="s">
+        <v>211</v>
+      </c>
+      <c r="S23" s="0" t="s">
+        <v>212</v>
+      </c>
+      <c r="T23" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="U23" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="V23" s="0" t="s">
         <v>70</v>
       </c>
-      <c r="AR20" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AS20" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O21" s="0" t="s">
-        <v>197</v>
-      </c>
-      <c r="P21" s="0" t="s">
-        <v>198</v>
-      </c>
-      <c r="Q21" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="R21" s="0" t="s">
-        <v>200</v>
-      </c>
-      <c r="S21" s="0" t="s">
-        <v>201</v>
-      </c>
-      <c r="T21" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="U21" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="V21" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="W21" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="X21" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="Y21" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="Z21" s="0" t="s">
+      <c r="W23" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="AB21" s="0" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O22" s="0" t="s">
-        <v>203</v>
-      </c>
-      <c r="P22" s="0" t="s">
-        <v>203</v>
-      </c>
-      <c r="Q22" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="R22" s="0" t="s">
-        <v>205</v>
-      </c>
-      <c r="S22" s="0" t="s">
-        <v>206</v>
-      </c>
-      <c r="T22" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="U22" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="V22" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="W22" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="X22" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="Y22" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="Z22" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="AB22" s="0" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O23" s="0" t="s">
-        <v>203</v>
-      </c>
-      <c r="P23" s="0" t="s">
-        <v>203</v>
-      </c>
-      <c r="Q23" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="R23" s="0" t="s">
-        <v>200</v>
-      </c>
-      <c r="S23" s="0" t="s">
-        <v>201</v>
-      </c>
-      <c r="T23" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="U23" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="V23" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="W23" s="0" t="s">
-        <v>68</v>
-      </c>
       <c r="X23" s="0" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="Y23" s="0" t="s">
-        <v>209</v>
+        <v>73</v>
       </c>
       <c r="Z23" s="0" t="s">
-        <v>210</v>
+        <v>74</v>
       </c>
       <c r="AB23" s="0" t="s">
-        <v>200</v>
-      </c>
-      <c r="AC23" s="0" t="s">
         <v>211</v>
       </c>
-      <c r="AD23" s="0" t="s">
-        <v>212</v>
-      </c>
-      <c r="AG23" s="0" t="s">
-        <v>203</v>
-      </c>
-      <c r="AH23" s="0" t="s">
-        <v>213</v>
-      </c>
-      <c r="AI23" s="0" t="s">
-        <v>213</v>
-      </c>
-      <c r="AJ23" s="0" t="s">
-        <v>209</v>
-      </c>
-      <c r="AK23" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AL23" s="0" t="s">
-        <v>91</v>
-      </c>
-      <c r="AN23" s="0" t="s">
-        <v>197</v>
-      </c>
-      <c r="AO23" s="0" t="s">
+    </row>
+    <row r="24" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N24" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="O24" s="0" t="s">
         <v>214</v>
       </c>
-      <c r="AP23" s="0" t="s">
+      <c r="P24" s="0" t="s">
         <v>214</v>
       </c>
-      <c r="AQ23" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="AR23" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AS23" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O24" s="0" t="s">
+      <c r="Q24" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="P24" s="0" t="s">
+      <c r="R24" s="0" t="s">
         <v>216</v>
       </c>
-      <c r="Q24" s="1" t="s">
+      <c r="S24" s="0" t="s">
         <v>217</v>
       </c>
-      <c r="R24" s="0" t="s">
+      <c r="T24" s="1" t="s">
         <v>218</v>
-      </c>
-      <c r="S24" s="0" t="s">
-        <v>219</v>
-      </c>
-      <c r="T24" s="1" t="s">
-        <v>220</v>
       </c>
       <c r="U24" s="0" t="n">
         <v>1</v>
       </c>
       <c r="V24" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="W24" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="X24" s="0" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="Y24" s="0" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="Z24" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="AA24" s="1" t="s">
-        <v>221</v>
+        <v>74</v>
       </c>
       <c r="AB24" s="0" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N25" s="0" t="s">
+        <v>64</v>
+      </c>
       <c r="O25" s="0" t="s">
+        <v>214</v>
+      </c>
+      <c r="P25" s="0" t="s">
+        <v>214</v>
+      </c>
+      <c r="Q25" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="P25" s="0" t="s">
-        <v>216</v>
-      </c>
-      <c r="Q25" s="1" t="s">
-        <v>217</v>
-      </c>
       <c r="R25" s="0" t="s">
-        <v>101</v>
+        <v>211</v>
       </c>
       <c r="S25" s="0" t="s">
-        <v>102</v>
+        <v>212</v>
       </c>
       <c r="T25" s="1" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="U25" s="0" t="n">
         <v>2</v>
       </c>
       <c r="V25" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="W25" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="X25" s="0" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="Y25" s="0" t="s">
-        <v>113</v>
+        <v>220</v>
       </c>
       <c r="Z25" s="0" t="s">
+        <v>221</v>
+      </c>
+      <c r="AB25" s="0" t="s">
+        <v>211</v>
+      </c>
+      <c r="AC25" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AD25" s="0" t="s">
+        <v>222</v>
+      </c>
+      <c r="AE25" s="0" t="s">
         <v>223</v>
       </c>
-      <c r="AB25" s="0" t="s">
-        <v>101</v>
-      </c>
-      <c r="AC25" s="0" t="s">
+      <c r="AH25" s="0" t="s">
+        <v>214</v>
+      </c>
+      <c r="AI25" s="0" t="s">
         <v>224</v>
       </c>
-      <c r="AG25" s="0" t="s">
-        <v>215</v>
-      </c>
-      <c r="AH25" s="0" t="s">
+      <c r="AJ25" s="0" t="s">
+        <v>224</v>
+      </c>
+      <c r="AK25" s="0" t="s">
+        <v>220</v>
+      </c>
+      <c r="AL25" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AM25" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN25" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AO25" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="AP25" s="0" t="s">
         <v>225</v>
       </c>
-      <c r="AJ25" s="0" t="s">
-        <v>113</v>
-      </c>
-      <c r="AK25" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AL25" s="0" t="s">
-        <v>91</v>
-      </c>
-      <c r="AN25" s="0" t="s">
-        <v>99</v>
-      </c>
-      <c r="AO25" s="0" t="s">
+      <c r="AQ25" s="0" t="s">
+        <v>225</v>
+      </c>
+      <c r="AR25" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="AS25" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AT25" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N26" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="O26" s="0" t="s">
         <v>226</v>
       </c>
-      <c r="AQ25" s="0" t="s">
+      <c r="P26" s="0" t="s">
+        <v>227</v>
+      </c>
+      <c r="Q26" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="R26" s="0" t="s">
+        <v>229</v>
+      </c>
+      <c r="S26" s="0" t="s">
+        <v>230</v>
+      </c>
+      <c r="T26" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="U26" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="V26" s="0" t="s">
         <v>70</v>
       </c>
-      <c r="AR25" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AS25" s="0" t="n">
+      <c r="W26" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="X26" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y26" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="Z26" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA26" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="AB26" s="0" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N27" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="O27" s="0" t="s">
+        <v>226</v>
+      </c>
+      <c r="P27" s="0" t="s">
+        <v>227</v>
+      </c>
+      <c r="Q27" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="R27" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="S27" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="T27" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="U27" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="V27" s="0" t="s">
+        <v>70</v>
+      </c>
+      <c r="W27" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="X27" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y27" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="Z27" s="0" t="s">
+        <v>234</v>
+      </c>
+      <c r="AB27" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="AC27" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AD27" s="0" t="s">
+        <v>235</v>
+      </c>
+      <c r="AH27" s="0" t="s">
+        <v>226</v>
+      </c>
+      <c r="AI27" s="0" t="s">
+        <v>236</v>
+      </c>
+      <c r="AK27" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="AL27" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AM27" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN27" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AO27" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="AP27" s="0" t="s">
+        <v>237</v>
+      </c>
+      <c r="AR27" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="AS27" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AT27" s="0" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O26" s="0" t="s">
-        <v>215</v>
-      </c>
-      <c r="P26" s="0" t="s">
+    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N28" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="O28" s="0" t="s">
+        <v>226</v>
+      </c>
+      <c r="P28" s="0" t="s">
+        <v>227</v>
+      </c>
+      <c r="Q28" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="R28" s="0" t="s">
         <v>216</v>
       </c>
-      <c r="Q26" s="1" t="s">
+      <c r="S28" s="0" t="s">
         <v>217</v>
       </c>
-      <c r="R26" s="0" t="s">
-        <v>205</v>
-      </c>
-      <c r="S26" s="0" t="s">
-        <v>206</v>
-      </c>
-      <c r="T26" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="U26" s="0" t="n">
+      <c r="T28" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="U28" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="V26" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="W26" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="X26" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="Y26" s="0" t="s">
-        <v>228</v>
-      </c>
-      <c r="Z26" s="0" t="s">
-        <v>229</v>
-      </c>
-      <c r="AB26" s="0" t="s">
-        <v>205</v>
-      </c>
-      <c r="AC26" s="0" t="s">
-        <v>230</v>
-      </c>
-      <c r="AG26" s="0" t="s">
-        <v>215</v>
-      </c>
-      <c r="AH26" s="0" t="s">
-        <v>225</v>
-      </c>
-      <c r="AJ26" s="0" t="s">
-        <v>228</v>
-      </c>
-      <c r="AK26" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AL26" s="0" t="s">
-        <v>91</v>
-      </c>
-      <c r="AN26" s="0" t="s">
-        <v>203</v>
-      </c>
-      <c r="AO26" s="0" t="s">
+      <c r="V28" s="0" t="s">
+        <v>70</v>
+      </c>
+      <c r="W28" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="X28" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y28" s="0" t="s">
+        <v>239</v>
+      </c>
+      <c r="Z28" s="0" t="s">
+        <v>240</v>
+      </c>
+      <c r="AB28" s="0" t="s">
+        <v>216</v>
+      </c>
+      <c r="AC28" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AD28" s="0" t="s">
+        <v>241</v>
+      </c>
+      <c r="AH28" s="0" t="s">
         <v>226</v>
       </c>
-      <c r="AQ26" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="AR26" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AS26" s="0" t="n">
+      <c r="AI28" s="0" t="s">
+        <v>236</v>
+      </c>
+      <c r="AK28" s="0" t="s">
+        <v>239</v>
+      </c>
+      <c r="AL28" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AM28" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN28" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="AO28" s="0" t="s">
+        <v>214</v>
+      </c>
+      <c r="AP28" s="0" t="s">
+        <v>237</v>
+      </c>
+      <c r="AR28" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="AS28" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="AT28" s="0" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AS20"/>
+  <autoFilter ref="A1:AT22"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>